<commit_message>
adjusted for PR feedback
</commit_message>
<xml_diff>
--- a/rules/CORE-000152/negative/01/data/unit-test-coreid-CG0265-negative 1.xlsx
+++ b/rules/CORE-000152/negative/01/data/unit-test-coreid-CG0265-negative 1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repos\Verisian\core-contributor\rules\CORE-000152\negative\01\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0112B810-3DD3-4E37-9467-FD638159AE2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD1F7747-68F1-4F38-AA81-85888E839056}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="203">
   <si>
     <t>Product</t>
   </si>
@@ -1077,8 +1077,11 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="5" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -1142,7 +1145,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B4" t="s">
         <v>6</v>
@@ -1151,13 +1154,13 @@
         <v>202</v>
       </c>
       <c r="D4">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E4" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -1174,15 +1177,15 @@
         <v>7</v>
       </c>
       <c r="E5" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F5" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B6" t="s">
         <v>6</v>
@@ -1191,18 +1194,18 @@
         <v>202</v>
       </c>
       <c r="D6">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="E6" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F6" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B7" t="s">
         <v>6</v>
@@ -1211,18 +1214,18 @@
         <v>202</v>
       </c>
       <c r="D7">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="E7" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="F7" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B8" t="s">
         <v>6</v>
@@ -1231,18 +1234,18 @@
         <v>202</v>
       </c>
       <c r="D8">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="E8" t="s">
         <v>20</v>
       </c>
       <c r="F8" t="s">
-        <v>134</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B9" t="s">
         <v>6</v>
@@ -1251,13 +1254,93 @@
         <v>202</v>
       </c>
       <c r="D9">
-        <v>35</v>
+        <v>20</v>
       </c>
       <c r="E9" t="s">
         <v>22</v>
       </c>
       <c r="F9" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" t="s">
+        <v>202</v>
+      </c>
+      <c r="D10">
+        <v>20</v>
+      </c>
+      <c r="E10" t="s">
+        <v>18</v>
+      </c>
+      <c r="F10" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>4</v>
+      </c>
+      <c r="B11" t="s">
+        <v>6</v>
+      </c>
+      <c r="C11" t="s">
+        <v>202</v>
+      </c>
+      <c r="D11">
+        <v>35</v>
+      </c>
+      <c r="E11" t="s">
+        <v>20</v>
+      </c>
+      <c r="F11" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>4</v>
+      </c>
+      <c r="B12" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" t="s">
+        <v>202</v>
+      </c>
+      <c r="D12">
+        <v>35</v>
+      </c>
+      <c r="E12" t="s">
+        <v>22</v>
+      </c>
+      <c r="F12" t="s">
         <v>51</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>4</v>
+      </c>
+      <c r="B13" t="s">
+        <v>6</v>
+      </c>
+      <c r="C13" t="s">
+        <v>202</v>
+      </c>
+      <c r="D13">
+        <v>35</v>
+      </c>
+      <c r="E13" t="s">
+        <v>18</v>
+      </c>
+      <c r="F13" t="s">
+        <v>132</v>
       </c>
     </row>
   </sheetData>
@@ -1453,7 +1536,7 @@
       <c r="C6" s="5">
         <v>1</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="6" t="s">
         <v>43</v>
       </c>
       <c r="F6" s="5" t="s">
@@ -1482,7 +1565,7 @@
       <c r="C7" s="5">
         <v>1</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="6" t="s">
         <v>49</v>
       </c>
       <c r="F7" s="5" t="s">
@@ -1808,7 +1891,7 @@
       <c r="C20" s="5">
         <v>1</v>
       </c>
-      <c r="E20" s="5" t="s">
+      <c r="E20" s="6" t="s">
         <v>90</v>
       </c>
       <c r="F20" s="5" t="s">
@@ -2171,7 +2254,7 @@
       <c r="C35" s="5">
         <v>1</v>
       </c>
-      <c r="E35" s="5" t="s">
+      <c r="E35" s="6" t="s">
         <v>132</v>
       </c>
       <c r="F35" s="5" t="s">

</xml_diff>